<commit_message>
Improve villa import edge cases
</commit_message>
<xml_diff>
--- a/villa-content-template.xlsx
+++ b/villa-content-template.xlsx
@@ -3742,7 +3742,7 @@
     <comment ref="A5" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -3819,7 +3819,7 @@
     <comment ref="A6" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -3854,7 +3854,7 @@
     <comment ref="A7" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -3889,7 +3889,7 @@
     <comment ref="A8" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -3924,7 +3924,7 @@
     <comment ref="A9" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -3959,7 +3959,7 @@
     <comment ref="A10" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -3994,7 +3994,7 @@
     <comment ref="A11" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -4029,7 +4029,7 @@
     <comment ref="A12" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -4064,7 +4064,7 @@
     <comment ref="A13" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -4099,7 +4099,7 @@
     <comment ref="A14" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -4134,7 +4134,7 @@
     <comment ref="A15" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -4169,7 +4169,7 @@
     <comment ref="A16" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -4204,7 +4204,7 @@
     <comment ref="A17" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -4239,7 +4239,7 @@
     <comment ref="A18" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -4274,7 +4274,7 @@
     <comment ref="A19" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -4309,7 +4309,7 @@
     <comment ref="A20" authorId="0">
       <text>
         <r>
-          <t>Optional. Example: 3 bedroom rate, 4 bedroom rate, Festive, or Winter.</t>
+          <t>Optional. Example: 3 Bedrooms, 4 Bedrooms, Festive, or Winter.</t>
         </r>
       </text>
     </comment>
@@ -4690,7 +4690,7 @@
     <t>Full Airbnb/Vrbo .ics URL supplied separately</t>
   </si>
   <si>
-    <t>Paste the full .ics/iCal calendar feed URL from Airbnb, Vrbo, or the owner calendar. The developer uses this after import to configure availability.</t>
+    <t>Paste one or more full .ics/iCal calendar feed URLs from Airbnb, Vrbo, or the owner calendar. Separate multiple URLs with a new line or note.</t>
   </si>
   <si>
     <t>postal_code</t>
@@ -5707,7 +5707,7 @@
     <t>generated_utc</t>
   </si>
   <si>
-    <t>2026-06-27T03:23:34.036Z</t>
+    <t>2026-06-28T00:32:45.270Z</t>
   </si>
 </sst>
 </file>
@@ -8002,7 +8002,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="21" ht="66" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" ht="60" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
         <v>111</v>
       </c>

</xml_diff>

<commit_message>
Refine villa importer amenity and nearby handling
</commit_message>
<xml_diff>
--- a/villa-content-template.xlsx
+++ b/villa-content-template.xlsx
@@ -1805,7 +1805,7 @@
     <comment ref="B5" authorId="0">
       <text>
         <r>
-          <t>Example: 10 minutes by car.</t>
+          <t>Example: 10 mins. The importer sorts these from shortest to longest.</t>
         </r>
       </text>
     </comment>
@@ -1840,7 +1840,7 @@
     <comment ref="B6" authorId="0">
       <text>
         <r>
-          <t>Example: 10 minutes by car.</t>
+          <t>Example: 10 mins. The importer sorts these from shortest to longest.</t>
         </r>
       </text>
     </comment>
@@ -1854,7 +1854,7 @@
     <comment ref="B7" authorId="0">
       <text>
         <r>
-          <t>Example: 10 minutes by car.</t>
+          <t>Example: 10 mins. The importer sorts these from shortest to longest.</t>
         </r>
       </text>
     </comment>
@@ -1868,7 +1868,7 @@
     <comment ref="B8" authorId="0">
       <text>
         <r>
-          <t>Example: 10 minutes by car.</t>
+          <t>Example: 10 mins. The importer sorts these from shortest to longest.</t>
         </r>
       </text>
     </comment>
@@ -1882,7 +1882,7 @@
     <comment ref="B9" authorId="0">
       <text>
         <r>
-          <t>Example: 10 minutes by car.</t>
+          <t>Example: 10 mins. The importer sorts these from shortest to longest.</t>
         </r>
       </text>
     </comment>
@@ -1896,7 +1896,7 @@
     <comment ref="B10" authorId="0">
       <text>
         <r>
-          <t>Example: 10 minutes by car.</t>
+          <t>Example: 10 mins. The importer sorts these from shortest to longest.</t>
         </r>
       </text>
     </comment>
@@ -1910,7 +1910,7 @@
     <comment ref="B11" authorId="0">
       <text>
         <r>
-          <t>Example: 10 minutes by car.</t>
+          <t>Example: 10 mins. The importer sorts these from shortest to longest.</t>
         </r>
       </text>
     </comment>
@@ -3207,7 +3207,7 @@
     <comment ref="A5" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3242,7 +3242,7 @@
     <comment ref="A6" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3256,7 +3256,7 @@
     <comment ref="A7" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3270,7 +3270,7 @@
     <comment ref="A8" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3284,7 +3284,7 @@
     <comment ref="A9" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3298,7 +3298,7 @@
     <comment ref="A10" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3312,7 +3312,7 @@
     <comment ref="A11" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3326,7 +3326,7 @@
     <comment ref="A12" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3340,7 +3340,7 @@
     <comment ref="A13" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3354,7 +3354,7 @@
     <comment ref="A14" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3368,7 +3368,7 @@
     <comment ref="A15" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3382,7 +3382,7 @@
     <comment ref="A16" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3396,7 +3396,7 @@
     <comment ref="A17" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3410,7 +3410,7 @@
     <comment ref="A18" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3424,7 +3424,7 @@
     <comment ref="A19" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3438,7 +3438,7 @@
     <comment ref="A20" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3452,7 +3452,7 @@
     <comment ref="A21" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3466,7 +3466,7 @@
     <comment ref="A22" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3480,7 +3480,7 @@
     <comment ref="A23" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3494,7 +3494,7 @@
     <comment ref="A24" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3508,7 +3508,7 @@
     <comment ref="A25" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3522,7 +3522,7 @@
     <comment ref="A26" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3536,7 +3536,7 @@
     <comment ref="A27" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3550,7 +3550,7 @@
     <comment ref="A28" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3564,7 +3564,7 @@
     <comment ref="A29" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3578,7 +3578,7 @@
     <comment ref="A30" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3592,7 +3592,7 @@
     <comment ref="A31" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3606,7 +3606,7 @@
     <comment ref="A32" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3620,7 +3620,7 @@
     <comment ref="A33" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3634,7 +3634,7 @@
     <comment ref="A34" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3648,7 +3648,7 @@
     <comment ref="A35" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3662,7 +3662,7 @@
     <comment ref="A36" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3676,7 +3676,7 @@
     <comment ref="A37" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3690,7 +3690,7 @@
     <comment ref="A38" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3704,7 +3704,7 @@
     <comment ref="A39" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -3718,7 +3718,7 @@
     <comment ref="A40" authorId="0">
       <text>
         <r>
-          <t>Choose a common group or type a clear alternative.</t>
+          <t>Choose Inside the Villa or Outdoor Living. Older custom groups are folded into the nearest section.</t>
         </r>
       </text>
     </comment>
@@ -4346,7 +4346,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1215" uniqueCount="454">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1211" uniqueCount="451">
   <si>
     <t>Barbados Escapes Villa Content Template</t>
   </si>
@@ -5233,7 +5233,7 @@
     <t>Amenities</t>
   </si>
   <si>
-    <t>Add one amenity per row and group similar items together. Keep in the order you would like to appear on the site.</t>
+    <t>Add one amenity per row. Use Inside the Villa or Outdoor Living; the importer always renders these as two sections.</t>
   </si>
   <si>
     <t>group</t>
@@ -5680,18 +5680,9 @@
     <t>Garden View</t>
   </si>
   <si>
-    <t>Services &amp; Staff</t>
-  </si>
-  <si>
     <t>Golf Course View</t>
   </si>
   <si>
-    <t>Technology &amp; Entertainment</t>
-  </si>
-  <si>
-    <t>Family Features</t>
-  </si>
-  <si>
     <t>schema_version</t>
   </si>
   <si>
@@ -5707,7 +5698,7 @@
     <t>generated_utc</t>
   </si>
   <si>
-    <t>2026-06-28T00:32:45.270Z</t>
+    <t>2026-06-28T00:53:38.387Z</t>
   </si>
 </sst>
 </file>
@@ -7495,7 +7486,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -7540,39 +7531,25 @@
         <v>316</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>440</v>
       </c>
       <c r="B4" t="s">
         <v>441</v>
       </c>
-      <c r="D4" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>442</v>
       </c>
       <c r="B5" t="s">
         <v>443</v>
       </c>
-      <c r="D5" t="s">
+    </row>
+    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
         <v>444</v>
-      </c>
-    </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
-        <v>445</v>
-      </c>
-      <c r="D6" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="7" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D7" t="s">
-        <v>447</v>
       </c>
     </row>
   </sheetData>
@@ -7588,26 +7565,26 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="B1" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="B2" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="B3" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add phase 1 villa search
Add responsive search controls and villa results filtering, extend villa data/import fields, and include the rebuilt Gutenberg assets.
</commit_message>
<xml_diff>
--- a/villa-content-template.xlsx
+++ b/villa-content-template.xlsx
@@ -23,7 +23,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Instructions'!$A1:$H25</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Overview'!$B1:$F23</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Overview'!$B1:$F25</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Villa Story'!$B1:$F25</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Nearby'!$A1:$F11</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Staff'!$A1:$H17</definedName>
@@ -2001,6 +2001,34 @@
         </r>
       </text>
     </comment>
+    <comment ref="D24" authorId="0">
+      <text>
+        <r>
+          <t>Example only. Type the new villa answer in the Client answer column.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F24" authorId="0">
+      <text>
+        <r>
+          <t>Optional client note. This is ignored by the importer.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D25" authorId="0">
+      <text>
+        <r>
+          <t>Example only. Type the new villa answer in the Client answer column.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F25" authorId="0">
+      <text>
+        <r>
+          <t>Optional client note. This is ignored by the importer.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -4603,12 +4631,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1291" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1319" uniqueCount="491">
   <si>
     <t>Barbados Escapes Villa Content Template</t>
   </si>
   <si>
-    <t>A simple content document for creating a new villa page accurately, with Monkey Hill shown as an example.</t>
+    <t>A simple content document for creating a new villa page and its search data accurately, with Monkey Hill shown as an example.</t>
   </si>
   <si>
     <t>How to use this template</t>
@@ -4737,7 +4765,7 @@
     <t>Villa Overview</t>
   </si>
   <si>
-    <t>Start with the core facts guests will see in the hero, villa card, specifications, and location section.</t>
+    <t>Start with the core facts used by the villa page, result cards, and search filters.</t>
   </si>
   <si>
     <t>Yellow = required   |   Blue = optional   |   Grey = fixed field   |   Red = skipped by import   |   Do not rename tabs</t>
@@ -4779,25 +4807,25 @@
     <t>property_area</t>
   </si>
   <si>
-    <t>Area or neighbourhood</t>
+    <t>Display area or neighbourhood</t>
   </si>
   <si>
     <t>Sugar Hill Resort</t>
   </si>
   <si>
-    <t>Example: Sugar Hill, Royal Westmoreland, or Gibbs.</t>
+    <t>Guest-facing copy. Example: Sugar Hill Resort, Royal Westmoreland, or Gibbs.</t>
   </si>
   <si>
     <t>parish</t>
   </si>
   <si>
-    <t>Villa location</t>
+    <t>Parish / broad location</t>
   </si>
   <si>
     <t>St. James</t>
   </si>
   <si>
-    <t>Choose an existing website location from the dropdown.</t>
+    <t>Choose the broad website location used for the address and taxonomy.</t>
   </si>
   <si>
     <t>hero_location_line</t>
@@ -4971,6 +4999,30 @@
     <t>Example: Sugar Hill Resort, St. James.</t>
   </si>
   <si>
+    <t>search_area</t>
+  </si>
+  <si>
+    <t>Search area</t>
+  </si>
+  <si>
+    <t>Sugar Hill Villas</t>
+  </si>
+  <si>
+    <t>Choose the exact enabled Area filter. This can differ from the guest-facing display area.</t>
+  </si>
+  <si>
+    <t>villa_collections</t>
+  </si>
+  <si>
+    <t>Search collections</t>
+  </si>
+  <si>
+    <t>Family Villas, Fully Staffed Villas, Ridgefront Villas, Villas with Community Gym, Villas with Pools</t>
+  </si>
+  <si>
+    <t>Optional. Separate chosen names with commas; leave blank for none. Options: Beachfront Villas; Family Villas; Fully Staffed Villas; Golf Resort Villas; Ridgefront Villas; Villas with Community Gym; Villas with Pools; Villas with Private Gym / Gym Equipment; Wedding Villas.</t>
+  </si>
+  <si>
     <t>Villa Story</t>
   </si>
   <si>
@@ -5970,30 +6022,72 @@
     <t>Amenity groups</t>
   </si>
   <si>
+    <t>Enabled search areas</t>
+  </si>
+  <si>
+    <t>Enabled villa collections</t>
+  </si>
+  <si>
     <t>Ocean View</t>
   </si>
   <si>
+    <t>Prospect</t>
+  </si>
+  <si>
+    <t>Beachfront Villas</t>
+  </si>
+  <si>
     <t>St. Peter</t>
   </si>
   <si>
     <t>Oceanfront</t>
   </si>
   <si>
+    <t>Royal Westmoreland Villas</t>
+  </si>
+  <si>
+    <t>Family Villas</t>
+  </si>
+  <si>
     <t>Mullins</t>
   </si>
   <si>
     <t>Hillside Retreat</t>
   </si>
   <si>
+    <t>Sandy Lane Villas</t>
+  </si>
+  <si>
+    <t>Fully Staffed Villas</t>
+  </si>
+  <si>
     <t>Paynes Bay</t>
   </si>
   <si>
     <t>Garden View</t>
   </si>
   <si>
+    <t>Golf Resort Villas</t>
+  </si>
+  <si>
     <t>Golf Course View</t>
   </si>
   <si>
+    <t>Ridgefront Villas</t>
+  </si>
+  <si>
+    <t>Villas with Community Gym</t>
+  </si>
+  <si>
+    <t>Villas with Pools</t>
+  </si>
+  <si>
+    <t>Villas with Private Gym / Gym Equipment</t>
+  </si>
+  <si>
+    <t>Wedding Villas</t>
+  </si>
+  <si>
     <t>schema_version</t>
   </si>
   <si>
@@ -6009,7 +6103,7 @@
     <t>generated_utc</t>
   </si>
   <si>
-    <t>2026-07-01T01:47:41.731Z</t>
+    <t>2026-08-03T21:12:24.919Z</t>
   </si>
 </sst>
 </file>
@@ -6634,6 +6728,7 @@
   <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
+    <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="8" width="18" customWidth="1"/>
   </cols>
@@ -6810,7 +6905,7 @@
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
     </row>
-    <row r="15" ht="34" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" ht="48" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>26</v>
       </c>
@@ -6996,7 +7091,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -7012,7 +7107,7 @@
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
@@ -7044,54 +7139,54 @@
     </row>
     <row r="4" ht="2" customHeight="1" hidden="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="B4" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="C4" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="D4" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="E4" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="30" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="D5" s="27" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="E5" s="27" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="F5" s="28" t="s">
         <v>51</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="I5" s="29" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="J5" s="29" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="K5" s="29" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="L5" s="29" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -7115,10 +7210,10 @@
         <v>54</v>
       </c>
       <c r="I6" s="34" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="J6" s="34" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="K6" s="26" t="s">
         <v>94</v>
@@ -7148,13 +7243,13 @@
         <v>54</v>
       </c>
       <c r="I7" s="34" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="J7" s="34" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="K7" s="26" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="L7" s="21">
         <v>7</v>
@@ -7181,13 +7276,13 @@
         <v>54</v>
       </c>
       <c r="I8" s="34" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="J8" s="34" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="K8" s="26" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="L8" s="21">
         <v>7</v>
@@ -7214,13 +7309,13 @@
         <v>54</v>
       </c>
       <c r="I9" s="34" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="J9" s="34" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="K9" s="26" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="L9" s="21">
         <v>14</v>
@@ -7645,7 +7740,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -7655,7 +7750,7 @@
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
@@ -7675,117 +7770,117 @@
     </row>
     <row r="4" ht="2" customHeight="1" hidden="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="B4" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="C5" s="28" t="s">
         <v>51</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="B6" s="20" t="s">
         <v>54</v>
       </c>
       <c r="C6" s="23"/>
       <c r="E6" s="21" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="F6" s="21" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="B7" s="20" t="s">
         <v>54</v>
       </c>
       <c r="C7" s="23"/>
       <c r="E7" s="21" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="35" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="B8" s="20" t="s">
         <v>54</v>
       </c>
       <c r="C8" s="23"/>
       <c r="E8" s="21" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="F8" s="21" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="35" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="B9" s="20" t="s">
         <v>54</v>
       </c>
       <c r="C9" s="23"/>
       <c r="E9" s="21" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="F9" s="21" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="35" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="B10" s="20" t="s">
         <v>54</v>
       </c>
       <c r="C10" s="23"/>
       <c r="E10" s="21" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="F10" s="21" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="35" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="B11" s="20" t="s">
         <v>54</v>
       </c>
       <c r="C11" s="23"/>
       <c r="E11" s="21" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="F11" s="21" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7797,10 +7892,10 @@
       </c>
       <c r="C12" s="23"/>
       <c r="E12" s="21" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="F12" s="21" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7882,7 +7977,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -7894,7 +7989,7 @@
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
@@ -7918,36 +8013,36 @@
     </row>
     <row r="4" ht="2" customHeight="1" hidden="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="B4" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="C4" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="30" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="C5" s="30" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="D5" s="28" t="s">
         <v>51</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
     </row>
     <row r="6" ht="54" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7962,13 +8057,13 @@
       </c>
       <c r="D6" s="23"/>
       <c r="F6" s="21" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="H6" s="21" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
     </row>
     <row r="7" ht="54" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7983,13 +8078,13 @@
       </c>
       <c r="D7" s="23"/>
       <c r="F7" s="21" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="H7" s="21" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
     </row>
     <row r="8" ht="54" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8004,13 +8099,13 @@
       </c>
       <c r="D8" s="23"/>
       <c r="F8" s="21" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="H8" s="21" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
     </row>
     <row r="9" ht="54" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8190,7 +8285,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>438</v>
+        <v>446</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -8198,7 +8293,7 @@
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>439</v>
+        <v>447</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
@@ -8219,13 +8314,13 @@
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
-        <v>440</v>
+        <v>448</v>
       </c>
       <c r="B5" s="28" t="s">
         <v>51</v>
       </c>
       <c r="D5" s="29" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -8234,7 +8329,7 @@
       </c>
       <c r="B6" s="23"/>
       <c r="D6" s="21" t="s">
-        <v>442</v>
+        <v>450</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -8243,7 +8338,7 @@
       </c>
       <c r="B7" s="23"/>
       <c r="D7" s="21" t="s">
-        <v>443</v>
+        <v>451</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -8252,7 +8347,7 @@
       </c>
       <c r="B8" s="23"/>
       <c r="D8" s="21" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
     </row>
   </sheetData>
@@ -8285,7 +8380,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -8293,7 +8388,7 @@
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
@@ -8309,16 +8404,16 @@
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
-        <v>447</v>
+        <v>455</v>
       </c>
       <c r="B4" s="27" t="s">
-        <v>448</v>
+        <v>456</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>449</v>
+        <v>457</v>
       </c>
       <c r="D4" s="27" t="s">
-        <v>450</v>
+        <v>458</v>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -8456,70 +8551,133 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="34" customWidth="1"/>
+    <col min="6" max="6" width="44" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
       <c r="B1" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
       <c r="C1" t="s">
-        <v>453</v>
+        <v>461</v>
       </c>
       <c r="D1" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <v>462</v>
+      </c>
+      <c r="E1" t="s">
+        <v>463</v>
+      </c>
+      <c r="F1" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>63</v>
       </c>
       <c r="B2" t="s">
-        <v>455</v>
+        <v>465</v>
       </c>
       <c r="C2" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="D2" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>328</v>
+      </c>
+      <c r="E2" t="s">
+        <v>466</v>
+      </c>
+      <c r="F2" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>456</v>
+        <v>468</v>
       </c>
       <c r="B3" t="s">
-        <v>457</v>
+        <v>469</v>
       </c>
       <c r="C3" t="s">
         <v>83</v>
       </c>
       <c r="D3" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>342</v>
+      </c>
+      <c r="E3" t="s">
+        <v>470</v>
+      </c>
+      <c r="F3" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>458</v>
+        <v>472</v>
       </c>
       <c r="B4" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>473</v>
+      </c>
+      <c r="E4" t="s">
+        <v>474</v>
+      </c>
+      <c r="F4" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>460</v>
+        <v>476</v>
       </c>
       <c r="B5" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
+        <v>477</v>
+      </c>
+      <c r="E5" t="s">
+        <v>216</v>
+      </c>
+      <c r="F5" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>462</v>
+        <v>479</v>
+      </c>
+      <c r="E6" t="s">
+        <v>124</v>
+      </c>
+      <c r="F6" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="7" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F7" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="8" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F8" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="9" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F9" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="10" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F10" t="s">
+        <v>484</v>
       </c>
     </row>
   </sheetData>
@@ -8532,29 +8690,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="50" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>463</v>
+        <v>485</v>
       </c>
       <c r="B1" t="s">
-        <v>464</v>
+        <v>486</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>465</v>
+        <v>487</v>
       </c>
       <c r="B2" t="s">
-        <v>466</v>
+        <v>488</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>467</v>
+        <v>489</v>
       </c>
       <c r="B3" t="s">
-        <v>468</v>
+        <v>490</v>
       </c>
     </row>
   </sheetData>
@@ -8569,7 +8731,7 @@
     <tabColor rgb="FFC4922A"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="9" hidden="1" customWidth="1"/>
@@ -8709,7 +8871,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" ht="46" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" ht="60" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
         <v>69</v>
       </c>
@@ -8809,7 +8971,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" ht="66" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" ht="88" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
         <v>85</v>
       </c>
@@ -8929,7 +9091,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" ht="66" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" ht="74" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="18" t="s">
         <v>107</v>
       </c>
@@ -9006,6 +9168,46 @@
         <v>121</v>
       </c>
       <c r="F23" s="23" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" ht="46" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="B24" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="D24" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="E24" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="F24" s="23" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="25" ht="100" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="B25" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="C25" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>128</v>
+      </c>
+      <c r="E25" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="F25" s="23" t="s">
         <v>54</v>
       </c>
     </row>
@@ -9016,7 +9218,7 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
   </mergeCells>
-  <dataValidations count="6">
+  <dataValidations count="7">
     <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Whole number required" error="Enter a whole number between 1 and 50." sqref="C10">
       <formula1>1</formula1>
       <formula2>50</formula2>
@@ -9034,6 +9236,9 @@
     </dataValidation>
     <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showErrorMessage="1" errorTitle="Positive USD amount required" error="Enter a positive USD amount. The $ symbol is accepted." sqref="C16">
       <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Choose or type a clear value" error="Select a suggested value or enter a clear alternative where permitted." sqref="C24">
+      <formula1>=Lists!$E$2:$E$6</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Choose or type a clear value" error="Select a suggested value or enter a clear alternative where permitted." sqref="C7">
       <formula1>=Lists!$A$2:$A$5</formula1>
@@ -9063,7 +9268,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -9073,7 +9278,7 @@
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
@@ -9113,219 +9318,219 @@
     </row>
     <row r="5" ht="46" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="C5" s="20" t="s">
         <v>54</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="E5" s="22" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="F5" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="6" ht="46" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" ht="60" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="C6" s="20" t="s">
         <v>54</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="F6" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="7" ht="46" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" ht="74" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C7" s="20" t="s">
         <v>54</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F7" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" ht="100" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>54</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="F8" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" ht="74" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>54</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="F9" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" ht="74" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="C10" s="20" t="s">
         <v>54</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="F10" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" ht="74" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>54</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="F11" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="12" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" ht="88" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>54</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="F12" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" ht="60" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="18" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>54</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="F13" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="14" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" ht="74" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="B14" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="C14" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="21" t="s">
+        <v>167</v>
+      </c>
+      <c r="E14" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="C14" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="D14" s="21" t="s">
-        <v>159</v>
-      </c>
-      <c r="E14" s="22" t="s">
-        <v>150</v>
-      </c>
       <c r="F14" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="15" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" ht="74" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>54</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="F15" s="23" t="s">
         <v>54</v>
@@ -9333,39 +9538,39 @@
     </row>
     <row r="16" ht="46" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="18" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="C16" s="20" t="s">
         <v>54</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="F16" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="17" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" ht="46" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="18" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="C17" s="20" t="s">
         <v>54</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="F17" s="23" t="s">
         <v>54</v>
@@ -9373,19 +9578,19 @@
     </row>
     <row r="18" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="18" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="C18" s="20" t="s">
         <v>54</v>
       </c>
       <c r="D18" s="21" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="F18" s="23" t="s">
         <v>54</v>
@@ -9393,19 +9598,19 @@
     </row>
     <row r="19" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="C19" s="20" t="s">
         <v>54</v>
       </c>
       <c r="D19" s="21" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="E19" s="22" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="F19" s="23" t="s">
         <v>54</v>
@@ -9413,19 +9618,19 @@
     </row>
     <row r="20" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="18" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="C20" s="24" t="s">
         <v>54</v>
       </c>
       <c r="D20" s="21" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="F20" s="23" t="s">
         <v>54</v>
@@ -9433,19 +9638,19 @@
     </row>
     <row r="21" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="C21" s="24" t="s">
         <v>54</v>
       </c>
       <c r="D21" s="21" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="F21" s="23" t="s">
         <v>54</v>
@@ -9453,59 +9658,59 @@
     </row>
     <row r="22" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="C22" s="20" t="s">
         <v>54</v>
       </c>
       <c r="D22" s="21" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="E22" s="22" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="F22" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="23" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" ht="100" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="C23" s="20" t="s">
         <v>54</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="F23" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="24" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" ht="74" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="18" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="C24" s="24" t="s">
         <v>54</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="E24" s="22" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="F24" s="23" t="s">
         <v>54</v>
@@ -9513,10 +9718,10 @@
     </row>
     <row r="25" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="C25" s="24" t="s">
         <v>54</v>
@@ -9525,7 +9730,7 @@
         <v>54</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="F25" s="23" t="s">
         <v>54</v>
@@ -9562,7 +9767,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -9572,7 +9777,7 @@
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
@@ -9612,119 +9817,119 @@
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="C5" s="20" t="s">
         <v>54</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="E5" s="22" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="F5" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" ht="60" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="C6" s="20" t="s">
         <v>54</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
       <c r="F6" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" ht="60" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>425</v>
+        <v>433</v>
       </c>
       <c r="C7" s="20" t="s">
         <v>54</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>426</v>
+        <v>434</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="F7" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="8" ht="46" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" ht="100" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>428</v>
+        <v>436</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>429</v>
+        <v>437</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>54</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="F8" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="9" ht="46" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" ht="88" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>433</v>
+        <v>441</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>54</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>434</v>
+        <v>442</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="F9" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="10" ht="46" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" ht="74" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>54</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="F10" s="23" t="s">
         <v>54</v>
@@ -9762,7 +9967,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -9772,7 +9977,7 @@
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
@@ -9792,27 +9997,27 @@
     </row>
     <row r="4" ht="2" customHeight="1" hidden="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="B4" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="C5" s="28" t="s">
         <v>51</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -9824,10 +10029,10 @@
       </c>
       <c r="C6" s="23"/>
       <c r="E6" s="21" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="F6" s="21" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -9839,10 +10044,10 @@
       </c>
       <c r="C7" s="23"/>
       <c r="E7" s="21" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -9854,10 +10059,10 @@
       </c>
       <c r="C8" s="23"/>
       <c r="E8" s="21" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="F8" s="21" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -9869,10 +10074,10 @@
       </c>
       <c r="C9" s="23"/>
       <c r="E9" s="21" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="F9" s="21" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -9884,10 +10089,10 @@
       </c>
       <c r="C10" s="23"/>
       <c r="E10" s="21" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="F10" s="21" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -9899,10 +10104,10 @@
       </c>
       <c r="C11" s="23"/>
       <c r="E11" s="21" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="F11" s="21" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -9939,7 +10144,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -9951,7 +10156,7 @@
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
@@ -9975,36 +10180,36 @@
     </row>
     <row r="4" ht="2" customHeight="1" hidden="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="B4" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="C4" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="30" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="C5" s="30" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="D5" s="28" t="s">
         <v>51</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10019,13 +10224,13 @@
       </c>
       <c r="D6" s="23"/>
       <c r="F6" s="21" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="H6" s="21" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10040,13 +10245,13 @@
       </c>
       <c r="D7" s="23"/>
       <c r="F7" s="21" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="H7" s="21" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10303,7 +10508,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -10325,7 +10530,7 @@
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
@@ -10369,81 +10574,81 @@
     </row>
     <row r="4" ht="2" customHeight="1" hidden="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="B4" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="C4" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="D4" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="E4" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="F4" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="G4" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="H4" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="C5" s="30" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="D5" s="27" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="E5" s="30" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="F5" s="30" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="G5" s="30" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="H5" s="30" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="I5" s="28" t="s">
         <v>51</v>
       </c>
       <c r="K5" s="29" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="L5" s="29" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="M5" s="29" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="N5" s="29" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="O5" s="29" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="P5" s="29" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="Q5" s="29" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="R5" s="29" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -10473,28 +10678,28 @@
       </c>
       <c r="I6" s="23"/>
       <c r="K6" s="21" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="L6" s="21" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="M6" s="21" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="N6" s="21" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="O6" s="21" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="P6" s="21" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="Q6" s="21" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="R6" s="21" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -10524,28 +10729,28 @@
       </c>
       <c r="I7" s="23"/>
       <c r="K7" s="21" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="L7" s="21" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="M7" s="21" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="N7" s="21" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="O7" s="21" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="P7" s="21" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="Q7" s="21" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="R7" s="21" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -10575,28 +10780,28 @@
       </c>
       <c r="I8" s="23"/>
       <c r="K8" s="21" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="L8" s="21" t="s">
+        <v>277</v>
+      </c>
+      <c r="M8" s="21" t="s">
+        <v>278</v>
+      </c>
+      <c r="N8" s="21" t="s">
+        <v>274</v>
+      </c>
+      <c r="O8" s="21" t="s">
+        <v>268</v>
+      </c>
+      <c r="P8" s="21" t="s">
         <v>269</v>
       </c>
-      <c r="M8" s="21" t="s">
-        <v>270</v>
-      </c>
-      <c r="N8" s="21" t="s">
-        <v>266</v>
-      </c>
-      <c r="O8" s="21" t="s">
-        <v>260</v>
-      </c>
-      <c r="P8" s="21" t="s">
-        <v>261</v>
-      </c>
       <c r="Q8" s="21" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="R8" s="21" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -10626,28 +10831,28 @@
       </c>
       <c r="I9" s="23"/>
       <c r="K9" s="21" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="L9" s="21" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="M9" s="21" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="N9" s="21" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="O9" s="21" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="P9" s="21" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="Q9" s="21" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="R9" s="21" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -10677,28 +10882,28 @@
       </c>
       <c r="I10" s="23"/>
       <c r="K10" s="21" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="L10" s="21" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="M10" s="21" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="N10" s="21" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="O10" s="21" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="P10" s="21" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="Q10" s="21" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="R10" s="21" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -10728,28 +10933,28 @@
       </c>
       <c r="I11" s="23"/>
       <c r="K11" s="21" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="L11" s="21" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="M11" s="21" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="N11" s="21" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="O11" s="21" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="P11" s="21" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="Q11" s="21" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="R11" s="21" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -10779,28 +10984,28 @@
       </c>
       <c r="I12" s="23"/>
       <c r="K12" s="21" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="L12" s="21" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="M12" s="21" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="N12" s="21" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="O12" s="21" t="s">
         <v>83</v>
       </c>
       <c r="P12" s="21" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="Q12" s="21" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="R12" s="21" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -10830,28 +11035,28 @@
       </c>
       <c r="I13" s="23"/>
       <c r="K13" s="21" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="L13" s="21" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="M13" s="21" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="N13" s="21" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="O13" s="21" t="s">
         <v>83</v>
       </c>
       <c r="P13" s="21" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="Q13" s="21" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="R13" s="21" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -11253,7 +11458,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -11264,7 +11469,7 @@
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
@@ -11303,47 +11508,47 @@
     </row>
     <row r="5" ht="46" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="B5" s="24" t="s">
         <v>54</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="E5" s="23" t="s">
         <v>54</v>
       </c>
       <c r="I5" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="B6" s="24" t="s">
         <v>54</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="E6" s="23" t="s">
         <v>54</v>
       </c>
       <c r="I6" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="31" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="B8" s="31"/>
       <c r="C8" s="31"/>
@@ -11355,7 +11560,7 @@
     </row>
     <row r="9" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="32" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="B9" s="32"/>
       <c r="C9" s="32"/>
@@ -11367,36 +11572,36 @@
     </row>
     <row r="10" ht="2" customHeight="1" hidden="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="B10" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="C10" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="B11" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="C11" s="30" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="D11" s="28" t="s">
         <v>51</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="F11" s="29" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -11411,13 +11616,13 @@
       </c>
       <c r="D12" s="23"/>
       <c r="E12" s="21" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="F12" s="21" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -11432,13 +11637,13 @@
       </c>
       <c r="D13" s="23"/>
       <c r="E13" s="21" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="F13" s="21" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -11453,13 +11658,13 @@
       </c>
       <c r="D14" s="23"/>
       <c r="E14" s="21" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="F14" s="21" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="G14" s="21" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -11601,7 +11806,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -11611,7 +11816,7 @@
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
@@ -11631,27 +11836,27 @@
     </row>
     <row r="4" ht="2" customHeight="1" hidden="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="B4" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="C5" s="28" t="s">
         <v>51</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11663,10 +11868,10 @@
       </c>
       <c r="C6" s="23"/>
       <c r="E6" s="21" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F6" s="21" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11678,10 +11883,10 @@
       </c>
       <c r="C7" s="23"/>
       <c r="E7" s="21" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11693,10 +11898,10 @@
       </c>
       <c r="C8" s="23"/>
       <c r="E8" s="21" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F8" s="21" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11708,10 +11913,10 @@
       </c>
       <c r="C9" s="23"/>
       <c r="E9" s="21" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F9" s="21" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11723,10 +11928,10 @@
       </c>
       <c r="C10" s="23"/>
       <c r="E10" s="21" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F10" s="21" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11738,10 +11943,10 @@
       </c>
       <c r="C11" s="23"/>
       <c r="E11" s="21" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F11" s="21" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11753,10 +11958,10 @@
       </c>
       <c r="C12" s="23"/>
       <c r="E12" s="21" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F12" s="21" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11768,10 +11973,10 @@
       </c>
       <c r="C13" s="23"/>
       <c r="E13" s="21" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F13" s="21" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11783,10 +11988,10 @@
       </c>
       <c r="C14" s="23"/>
       <c r="E14" s="21" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F14" s="21" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11798,10 +12003,10 @@
       </c>
       <c r="C15" s="23"/>
       <c r="E15" s="21" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F15" s="21" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11813,10 +12018,10 @@
       </c>
       <c r="C16" s="23"/>
       <c r="E16" s="21" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F16" s="21" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
     </row>
     <row r="17" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11828,10 +12033,10 @@
       </c>
       <c r="C17" s="23"/>
       <c r="E17" s="21" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11843,10 +12048,10 @@
       </c>
       <c r="C18" s="23"/>
       <c r="E18" s="21" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F18" s="21" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
     </row>
     <row r="19" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11858,10 +12063,10 @@
       </c>
       <c r="C19" s="23"/>
       <c r="E19" s="21" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="F19" s="21" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11873,10 +12078,10 @@
       </c>
       <c r="C20" s="23"/>
       <c r="E20" s="21" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="F20" s="21" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11888,10 +12093,10 @@
       </c>
       <c r="C21" s="23"/>
       <c r="E21" s="21" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="F21" s="21" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11903,10 +12108,10 @@
       </c>
       <c r="C22" s="23"/>
       <c r="E22" s="21" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="F22" s="21" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
     </row>
     <row r="23" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11918,10 +12123,10 @@
       </c>
       <c r="C23" s="23"/>
       <c r="E23" s="21" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="F23" s="21" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
     </row>
     <row r="24" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11933,10 +12138,10 @@
       </c>
       <c r="C24" s="23"/>
       <c r="E24" s="21" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="F24" s="21" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
     </row>
     <row r="25" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11948,10 +12153,10 @@
       </c>
       <c r="C25" s="23"/>
       <c r="E25" s="21" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="F25" s="21" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
     </row>
     <row r="26" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11963,10 +12168,10 @@
       </c>
       <c r="C26" s="23"/>
       <c r="E26" s="21" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="F26" s="21" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
     </row>
     <row r="27" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11978,10 +12183,10 @@
       </c>
       <c r="C27" s="23"/>
       <c r="E27" s="21" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="F27" s="21" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
     </row>
     <row r="28" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -11993,10 +12198,10 @@
       </c>
       <c r="C28" s="23"/>
       <c r="E28" s="21" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="F28" s="21" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
     </row>
     <row r="29" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat: add villa guest age policies
</commit_message>
<xml_diff>
--- a/villa-content-template.xlsx
+++ b/villa-content-template.xlsx
@@ -23,7 +23,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Instructions'!$A1:$H25</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Overview'!$B1:$F25</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Overview'!$B1:$F26</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Villa Story'!$B1:$F25</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Nearby'!$A1:$F11</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Staff'!$A1:$H17</definedName>
@@ -8551,7 +8551,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="24" customWidth="1"/>
@@ -8559,6 +8559,7 @@
     <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="5" width="34" customWidth="1"/>
     <col min="6" max="6" width="44" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -8579,6 +8580,26 @@
       </c>
       <c r="F1" t="s">
         <v>464</v>
+      </c>
+      <c r="G1" s="0" t="inlineStr">
+        <is>
+          <t>Guest age policy</t>
+        </is>
+      </c>
+      <c r="G2" s="0" t="inlineStr">
+        <is>
+          <t>All ages</t>
+        </is>
+      </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t>Ages 12+ only</t>
+        </is>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t>Adults 18+ only</t>
+        </is>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -8731,7 +8752,7 @@
     <tabColor rgb="FFC4922A"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="9" hidden="1" customWidth="1"/>
@@ -9211,6 +9232,38 @@
         <v>54</v>
       </c>
     </row>
+    <row r="26" ht="54" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>guest_age_policy</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Guest age policy</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>All ages</t>
+        </is>
+      </c>
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>All ages</t>
+        </is>
+      </c>
+      <c r="E26" s="22" t="inlineStr">
+        <is>
+          <t>Choose All ages, Ages 12+ only, or Adults 18+ only. Leave as All ages when there is no age restriction.</t>
+        </is>
+      </c>
+      <c r="F26" s="23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="B4:F4"/>
   <mergeCells count="3">
@@ -9218,7 +9271,10 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
   </mergeCells>
-  <dataValidations count="7">
+  <dataValidations count="8">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Choose a guest age policy" error="Select All ages, Ages 12+ only, or Adults 18+ only." sqref="C26">
+      <formula1>=Lists!$G$2:$G$4</formula1>
+    </dataValidation>
     <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Whole number required" error="Enter a whole number between 1 and 50." sqref="C10">
       <formula1>1</formula1>
       <formula2>50</formula2>

</xml_diff>